<commit_message>
fix: corrigir placar de Chengdu 2x1 como GREEN e atualizar lucro para +6.79u
</commit_message>
<xml_diff>
--- a/metodos_aprovados/Sinais_Metodos_Aprovados_2026-08-29.xlsx
+++ b/metodos_aprovados/Sinais_Metodos_Aprovados_2026-08-29.xlsx
@@ -576,22 +576,22 @@
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>2x2</t>
+          <t>2x1</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>RED</t>
+          <t>GREEN</t>
         </is>
       </c>
       <c r="H3" t="n">
         <v>10.06</v>
       </c>
       <c r="I3" t="n">
-        <v>-50</v>
+        <v>9.609999999999999</v>
       </c>
       <c r="J3" t="n">
-        <v>-4.97</v>
+        <v>0.955</v>
       </c>
       <c r="K3" t="inlineStr">
         <is>
@@ -599,7 +599,7 @@
         </is>
       </c>
       <c r="L3" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="M3" t="n">
         <v>1.39</v>

</xml_diff>